<commit_message>
repalce the excel with the updated
</commit_message>
<xml_diff>
--- a/user_feedback/dMessage FeedBack  (Responses).xlsx
+++ b/user_feedback/dMessage FeedBack  (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="198">
   <si>
     <t>Timestamp</t>
   </si>
@@ -266,6 +266,345 @@
   </si>
   <si>
     <t>As a new user its been a struggle to get started - a start here guide would help. QR codes to look up usernames would make finding people easier. Delivery indicators and read receipts are basic features missing.</t>
+  </si>
+  <si>
+    <t>GBLKEU6IAQIV6Z4YS6CCWIKDOL2WA6CHLL5WPQH4ES47HRHZ2TLUOMF2</t>
+  </si>
+  <si>
+    <t>angle.dmessage@gmail.com</t>
+  </si>
+  <si>
+    <t>Angle</t>
+  </si>
+  <si>
+    <t>It was the best one out there</t>
+  </si>
+  <si>
+    <t>GC7KQY5DRQH4YNMZXDEQ4V2XZ5UJG2YLSILQRLI5SCNQBTEMP2XEWZSQ</t>
+  </si>
+  <si>
+    <t>aaron664@gmail.com</t>
+  </si>
+  <si>
+    <t>Aaron</t>
+  </si>
+  <si>
+    <t>I'm really enjoying the end-to-end encryption on dMessage, it's great to know my conversations are secure. One thing that's been frustrating is the onboarding process, it takes a while to set up a Stellar wallet and fund it with testnet lumens just to try out the app - maybe consider adding a simpler way to get started with a temporary test account or something.</t>
+  </si>
+  <si>
+    <t>GDUKNDRHLOBAODTLEWMUGQSDU4IHMWE3G6U2P3VVSY5UUHCEXMW5NSUA</t>
+  </si>
+  <si>
+    <t>abe124@gmail.com</t>
+  </si>
+  <si>
+    <t>Abe</t>
+  </si>
+  <si>
+    <t>Loving the E2E encryption on dMessage, especially while testing things out on the Stellar testnet! The only downside right now is not being able to search through chats. It's tough trying to find specific messages or old threads, so adding a search bar would be a massive upgrade for usability.</t>
+  </si>
+  <si>
+    <t>GAKTAMLOF3DFMS2OAHJEAB7LBVEXAN6AE4LETYWDJMNINYGVX6NU2PKR</t>
+  </si>
+  <si>
+    <t>abiel35@gmail.com</t>
+  </si>
+  <si>
+    <t>Abiel</t>
+  </si>
+  <si>
+    <t>I've been using dMessage on Stellar testnet for a while now and I'm impressed with how seamless the file sharing feature is, it's really convenient to send and receive files directly on the app. However, I think the onboarding process could be improved, it took me a while to understand how to register a username and I had to search for tutorials online, maybe adding a more detailed guide or walkthrough during the initial setup would make it easier for new users like I was.</t>
+  </si>
+  <si>
+    <t>GCV5226FBC4FC3WXSIGQOPQBV2BPAHFLPSSORGEAUSFGSVUNGEEWLGKW</t>
+  </si>
+  <si>
+    <t>abigail769@gmail.com</t>
+  </si>
+  <si>
+    <t>Abigail</t>
+  </si>
+  <si>
+    <t>I'm really enjoying the end-to-end encryption on dMessage, it gives me peace of mind when sending sensitive information to friends and family. One thing that's been frustrating is the lack of a search function in group chats, it can be really hard to find specific messages or files that were sent a while ago.</t>
+  </si>
+  <si>
+    <t>GDACACZH7X2G2KUJMX6VV3UZ3IBNPIWSCFHTKEK5P5H2G7TIXED4NIEN</t>
+  </si>
+  <si>
+    <t>acelle152@gmail.com</t>
+  </si>
+  <si>
+    <t>Acelle</t>
+  </si>
+  <si>
+    <t>I'm really enjoying using dMessage so far, especially the QR code feature for adding new contacts, it's so much easier than typing out a long stellar wallet address. One thing I wish they would improve is the search functionality within the contact list, it can be pretty slow and frustrating to find a specific conversation when you have a lot of contacts, it would be great if they could speed up the loading times for this feature.</t>
+  </si>
+  <si>
+    <t>GBX2YHDKYTPCDT23K4BXP7YTHVCD5RMX2T2IA4VRZBO5RCFX2PY6TUO2</t>
+  </si>
+  <si>
+    <t>adiel764@gmail.com</t>
+  </si>
+  <si>
+    <t>Adiel</t>
+  </si>
+  <si>
+    <t>I'm really enjoying the end-to-end encryption feature on dMessage, it's a major selling point for me as I feel my conversations are truly private. However, I wish the onboarding process was smoother - I had to manually add each contact by entering their Stellar wallet address, a QR code scanner would've made this process a lot easier.</t>
+  </si>
+  <si>
+    <t>GA7W7GLSURIQPNK3QQ2FG5YZ4Z6MM4AZ2JO5AMVKZML54XNJP7ZQ6T6X</t>
+  </si>
+  <si>
+    <t>adrana114@gmail.com</t>
+  </si>
+  <si>
+    <t>Adrana</t>
+  </si>
+  <si>
+    <t>I'm really enjoying using dMessage so far, especially the end-to-end encryption feature which gives me peace of mind when sending sensitive messages. One thing that I think could be improved is the onboarding process - it took me a few minutes to figure out how to register a username and I think a more guided tutorial would be helpful for new users like me.</t>
+  </si>
+  <si>
+    <t>GA3YQ5HIZOLOP7GZEJCGRZODHL5C2G4VZNEOODVMJHVTISF4XQUZ23TY</t>
+  </si>
+  <si>
+    <t>adrian702@gmail.com</t>
+  </si>
+  <si>
+    <t>Adrian</t>
+  </si>
+  <si>
+    <t>I really like how seamless the onboarding process is in dMessage, the QR code scan to link my Stellar testnet wallet was quick and easy. One thing that could be improved is the search functionality, sometimes it takes a few seconds for results to load and it would be great if I could search for messages within a specific chat or group, currently it only searches my entire contact list.</t>
+  </si>
+  <si>
+    <t>GCGS7S2Z2365KKLBHDIQM4VKYDTZ6SDMHRQQFPWHS7YMIRNV5IW6HEI6</t>
+  </si>
+  <si>
+    <t>adriana768@gmail.com</t>
+  </si>
+  <si>
+    <t>Adriana</t>
+  </si>
+  <si>
+    <t>I've been testing dMessage on Stellar testnet and I have to say the end-to-end encryption gives me a lot of confidence in the security of my conversations, it's great to see this level of focus on user privacy. One thing that could be improved is the onboarding process - I found it a bit confusing to register a username and set up my account, a more guided tutorial or clearer instructions would have been really helpful.</t>
+  </si>
+  <si>
+    <t>GBNPM6NYBRQJ5XAIBEZ7ZFTHKOTSYROSFGKT47EH2YVNL54PXHFS6SM4</t>
+  </si>
+  <si>
+    <t>aera923@gmail.com</t>
+  </si>
+  <si>
+    <t>Aera</t>
+  </si>
+  <si>
+    <t>I really like how seamless the onboarding process was for dMessage, the QR code scanning made it super easy to connect my Stellar wallet and get started right away. However, I think it would be really useful to have a search function within conversations, I had a bit of trouble finding a specific message in a group chat I was in, it took a while to scroll through.</t>
+  </si>
+  <si>
+    <t>GCNDZKIMYGREDSS2VCS4SGAFUI6XYNRSWPOD4NHFM23WN6XFNUQLRZMT</t>
+  </si>
+  <si>
+    <t>aidan568@gmail.com</t>
+  </si>
+  <si>
+    <t>Aidan</t>
+  </si>
+  <si>
+    <t>I've been testing dMessage on Stellar testnet and I have to say, the end-to-end encryption feature gives me a lot of confidence in the security of my messages, which is a major plus. One thing that's been frustrating me though is the lack of a search function, I've been trying to find a specific conversation from a few days ago and it's been a real pain to scroll through all my chats to find it.</t>
+  </si>
+  <si>
+    <t>GCHSUWLHR45T7BTPJREG6AM7FTQ63QJXGO366LKRL3Z25AO374EFDCML</t>
+  </si>
+  <si>
+    <t>aiesha99@gmail.com</t>
+  </si>
+  <si>
+    <t>Aiesha</t>
+  </si>
+  <si>
+    <t>I've been playing around with dMessage and I really love how seamless the username registration process is, it's so easy to get started and find friends to chat with. One thing that's been frustrating is the loading times when sending files, it takes a while for them to upload and it would be great if this could be sped up.</t>
+  </si>
+  <si>
+    <t>GAVV7U6KYNNKWOVAV2E24PGWSUY33DL47H5AVMKDPN5G3ZSC35UISXL6</t>
+  </si>
+  <si>
+    <t>aira614@gmail.com</t>
+  </si>
+  <si>
+    <t>Aira</t>
+  </si>
+  <si>
+    <t>I'm really enjoying using dMessage on Stellar testnet, especially the seamless username registration process that allows me to easily find and connect with friends. However, I wish the app had a more robust search function, as it's currently a bit tedious to scroll through my entire contact list to find a specific conversation.</t>
+  </si>
+  <si>
+    <t>GD3NA7WACXGBNMFHJOMU6EMBNCH3Y7UEJAPXRE4PZRBFS33S34ELN5ML</t>
+  </si>
+  <si>
+    <t>aireen442@gmail.com</t>
+  </si>
+  <si>
+    <t>Aireen</t>
+  </si>
+  <si>
+    <t>I really like how seamless the QR code scanning is for adding new contacts on dMessage, it makes onboarding friends so much easier. One thing that could be improved is the loading times when sending images, it takes a bit too long and sometimes I'm not even sure if the file has gone through.</t>
+  </si>
+  <si>
+    <t>GC7D65277ISRCXU6AOFGJA4PV6DV4HQWTCLUIPZKB664MS3JNGZI6I6A</t>
+  </si>
+  <si>
+    <t>alea37@gmail.com</t>
+  </si>
+  <si>
+    <t>Alea</t>
+  </si>
+  <si>
+    <t>I like the idea of decentralized messaging but the onboarding needs work. A quick tutorial when you first log in would help a lot. Also QR code support for sharing wallet addresses would make connecting with others much easier.</t>
+  </si>
+  <si>
+    <t>GAG4EJQ6F4EMR2RABC6NM5IRLEO3GIOPN5FXH2K46FD4EDTVZWTGKH6Z</t>
+  </si>
+  <si>
+    <t>alexa584@gmail.com</t>
+  </si>
+  <si>
+    <t>Alexa</t>
+  </si>
+  <si>
+    <t>I really like how seamless the username registration process is on dMessage, it's so easy to create a unique handle and start chatting right away. One thing that's been frustrating for me is the lack of a search function in group chats, it can be hard to find specific messages or threads when the conversation gets going.</t>
+  </si>
+  <si>
+    <t>GAJPQOMZEWHAMOON5A4HPUOXUZ7U5XF3FZYGPS2XZADKIAGMLJG7NJSQ</t>
+  </si>
+  <si>
+    <t>alexander213@gmail.com</t>
+  </si>
+  <si>
+    <t>Alexander</t>
+  </si>
+  <si>
+    <t>I've been testing dMessage on Stellar testnet for a while now and I have to say the end-to-end encryption feature is really impressive, it's great to know my conversations are secure. However, I wish the contact list loading times were faster, sometimes it takes a few seconds to load all my contacts which can be frustrating when I'm in a hurry to send a message.</t>
+  </si>
+  <si>
+    <t>GAASYNT3PLXVLZET6SUGC246NFLK22I25N5SS2NFUIFYV56NBEYEOF4G</t>
+  </si>
+  <si>
+    <t>alexis743@gmail.com</t>
+  </si>
+  <si>
+    <t>Alexis</t>
+  </si>
+  <si>
+    <t>I really like how seamless the username registration process is on dMessage, it's a huge plus that I can easily create a unique handle for myself without having to deal with complicated public key management. One area that could use improvement is the search function - I found it a bit finicky when trying to look up specific conversations or contacts, sometimes it wouldn't pull up results even when I knew the exact name.</t>
+  </si>
+  <si>
+    <t>GCCCOCSEG46S5RWWSTIXFPNREPJHBZT3RB4C7R2GSMQJW64FJLWHM4YT</t>
+  </si>
+  <si>
+    <t>ali728@gmail.com</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>I'm really enjoying using dMessage on Stellar testnet so far, especially the end-to-end encryption which gives me peace of mind when sending sensitive information. One thing that could be improved is the onboarding process, I found it a bit confusing to set up my account and had to retry a few times before I got it right, maybe adding a guided tour or more instructions would help new users like I was.</t>
+  </si>
+  <si>
+    <t>GAMAVJ5S4F5JUKGEJJ3A3FQQRBQRN7ZKT6VP4XTKCMEN7MY4HU3B6UHG</t>
+  </si>
+  <si>
+    <t>aliana568@gmail.com</t>
+  </si>
+  <si>
+    <t>Aliana</t>
+  </si>
+  <si>
+    <t>I've been using dMessage on Stellar testnet and I really like the end-to-end encryption feature, it makes me feel secure sending messages to my friends. One thing that could be improved is the onboarding process - it took me a few tries to register a username, it would be great if there were clearer instructions or a walkthrough to help new users get started.</t>
+  </si>
+  <si>
+    <t>GCMRLVCLG642LJJVU5GNHSRF4M37QSPZXF6UOQSU3LWKZWQQSSUFCV62</t>
+  </si>
+  <si>
+    <t>alianna439@gmail.com</t>
+  </si>
+  <si>
+    <t>Alianna</t>
+  </si>
+  <si>
+    <t>I'm really enjoying the end-to-end encryption feature in dMessage, it gives me peace of mind knowing my messages are secure. One thing that could be improved is the onboarding process - I found it a bit confusing to register my username, maybe adding a more detailed guide or a tutorial would help new users like I was.</t>
+  </si>
+  <si>
+    <t>GCTZMYZUOFHQP5OQ7AWXHNGSX2KPMXIC2TTSJQSYEE7MWOJWFK3V3PY2</t>
+  </si>
+  <si>
+    <t>alice235@gmail.com</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>I've been using dMessage on Stellar testnet and I love how seamless the onboarding process is, especially with the QR code login feature that makes it easy to connect my Stellar wallet. However, I wish there was a more intuitive way to manage my contact list, perhaps with the ability to search for specific usernames or add people to a favorites list, as it can get cluttered quickly with all the testnet users.</t>
+  </si>
+  <si>
+    <t>GCJHF4GGEXDQO2NITG4AXDWCROLIU4SACOZ5RJYEMAJLL2ZEO5HGQ66I</t>
+  </si>
+  <si>
+    <t>aljohn469@gmail.com</t>
+  </si>
+  <si>
+    <t>Aljohn</t>
+  </si>
+  <si>
+    <t>I've been using dMessage on Stellar testnet for a while now and I have to say the end-to-end encryption feature gives me a lot of confidence in the security of my messages, it's great that my conversations are protected from prying eyes. One thing that could be improved is the onboarding process, it took me a few attempts to register a username and set up my account, it would be great if there were more guidance throughout the process.</t>
+  </si>
+  <si>
+    <t>GBB5PLY5OD3IPS3MZ3O7YF6LCF3IMYHMQ7XGIHZ562KTI7OFRZF6VLJV</t>
+  </si>
+  <si>
+    <t>allaneo613@gmail.com</t>
+  </si>
+  <si>
+    <t>Allaneo</t>
+  </si>
+  <si>
+    <t>I'm really enjoying the seamless onboarding process of dMessage, it's incredibly easy to set up and start chatting with friends using the Stellar testnet. One thing that could be improved is the loading times when sending large files - I've noticed it can take up to 10 seconds for the file to be fully transmitted, which can be frustrating.</t>
+  </si>
+  <si>
+    <t>GBTH76C4WRTO6PDBJLIOMDV7NR4FQ4RMEJ67IRCNUVLBQNXHN6OVBB6T</t>
+  </si>
+  <si>
+    <t>alliah294@gmail.com</t>
+  </si>
+  <si>
+    <t>Alliah</t>
+  </si>
+  <si>
+    <t>I love how seamless the onboarding process is for dMessage, especially the use of QR codes to easily add contacts, it makes getting started a breeze. However, I do wish there was a dark mode option to reduce eye strain, especially when using the app for extended periods of time.</t>
+  </si>
+  <si>
+    <t>GDV3HR5ZN2LWDLOJK5RMJFXCFNMY4DLD7SEO7TCWCK372GZZ4PC5G5TF</t>
+  </si>
+  <si>
+    <t>allysha838@gmail.com</t>
+  </si>
+  <si>
+    <t>Allysha</t>
+  </si>
+  <si>
+    <t>I'm really enjoying using dMessage so far, the end-to-end encryption gives me peace of mind when chatting with friends and family, but I wish the onboarding process was a bit smoother - it took me a few tries to successfully register my username and I had to manually add the public key.</t>
+  </si>
+  <si>
+    <t>GBZT4OTRR66HRSVQG62TNHLD6PNCRH2EDS3PSKAFXIWCHG7CDIO3H3AU</t>
+  </si>
+  <si>
+    <t>allyssa900@gmail.com</t>
+  </si>
+  <si>
+    <t>Allyssa</t>
+  </si>
+  <si>
+    <t>I love that dMessage uses end-to-end encryption, it makes me feel secure when sending sensitive information to my friends. However, I think the onboarding process could be improved, it took me a while to understand how to register my username and claim my Stellar testnet account, maybe a more detailed tutorial would be helpful.</t>
+  </si>
+  <si>
+    <t>I love how seamless the onboarding process is on dMessage, it's super easy to register a username and start chatting right away, but I think the app could really benefit from implementing read receipts so I can see when my friends have actually read my messages, it's a pretty standard feature that's missing right now.</t>
   </si>
 </sst>
 </file>
@@ -400,7 +739,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E21" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E50" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="5">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="1. Wallet Address" id="2"/>
@@ -975,6 +1314,499 @@
         <v>84</v>
       </c>
     </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="4">
+        <v>46202.95416298611</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="4">
+        <v>46202.95908930556</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="4">
+        <v>46202.96155907407</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="4">
+        <v>46202.98651728009</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="4">
+        <v>46202.98662998843</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="4">
+        <v>46202.99050594907</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="4">
+        <v>46202.990655393514</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="4">
+        <v>46202.99077244213</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="4">
+        <v>46202.99089748843</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="4">
+        <v>46202.99125917824</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="4">
+        <v>46202.99139016204</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="4">
+        <v>46202.99172196759</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="4">
+        <v>46202.99402186343</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="4">
+        <v>46202.99412379629</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="4">
+        <v>46202.994207592594</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="4">
+        <v>46202.99560408565</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="4">
+        <v>46202.99572980324</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="A39" s="4">
+        <v>46202.995818310184</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="40" ht="22.5" customHeight="1">
+      <c r="A40" s="4">
+        <v>46202.99594206018</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="41" ht="22.5" customHeight="1">
+      <c r="A41" s="4">
+        <v>46202.99691386574</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="42" ht="22.5" customHeight="1">
+      <c r="A42" s="4">
+        <v>46202.99702271991</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="43" ht="22.5" customHeight="1">
+      <c r="A43" s="4">
+        <v>46202.99711847222</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="44" ht="22.5" customHeight="1">
+      <c r="A44" s="4">
+        <v>46202.99723569445</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="45" ht="22.5" customHeight="1">
+      <c r="A45" s="4">
+        <v>46202.99840575231</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1">
+      <c r="A46" s="4">
+        <v>46202.99858381944</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="47" ht="22.5" customHeight="1">
+      <c r="A47" s="4">
+        <v>46202.998682418984</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="48" ht="22.5" customHeight="1">
+      <c r="A48" s="4">
+        <v>46202.998789317135</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="49" ht="22.5" customHeight="1">
+      <c r="A49" s="4">
+        <v>46202.998904189815</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" ht="22.5" customHeight="1">
+      <c r="A50" s="4">
+        <v>46202.999103090275</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>